<commit_message>
Input citations using Zotero. Deleteded separate references page as references are at the bottom of each page.
</commit_message>
<xml_diff>
--- a/administrative-database-guidance/data/tbl_summary_administrative_datasets.xlsx
+++ b/administrative-database-guidance/data/tbl_summary_administrative_datasets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MikaylaBoginsky\Documents\technicalguide\administrative-database-guidance\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A73A0A56-5D64-4E9A-B7D2-FD4318C8F94E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C94780C7-913B-476C-BBBB-D61144DA5466}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9090" yWindow="345" windowWidth="18015" windowHeight="14715" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
     <t>Administrative dataset</t>
   </si>
@@ -31,48 +31,18 @@
     <t>Key variables</t>
   </si>
   <si>
-    <t>Years available</t>
-  </si>
-  <si>
     <t>Unit of observation</t>
   </si>
   <si>
-    <t>Access/Governance</t>
-  </si>
-  <si>
-    <t>Major limitations</t>
-  </si>
-  <si>
     <t>National pupil database (NPD)</t>
   </si>
   <si>
-    <t>Children who attended school in England</t>
-  </si>
-  <si>
     <t>Attainment data (KS1-5), absence, exclusions and children’s social care data.</t>
   </si>
   <si>
-    <t>School census (2001/02 to 2025/26)
-Key Stage 1 (1997/98 to 2022/23)
-Key Stage 2 (1995/98 to 2024/25)
-Key Stage 3 (1997/98 to 2012/13)
-Key Stage 4 (2001/02 to 2024/25)
-Key Stage 5 (2001/02 to 2024/25)
-Absences and exclusions (2005/06 to 2024/25)
-Children looked after (2005/06 to 2024/25)
-Children in Need (2008/09 to 2024/25)</t>
-  </si>
-  <si>
     <t>Individual-level and school level (not class level).</t>
   </si>
   <si>
-    <t>Managed by the Department for Education (DfE). Access is highly restricted and requires submitting an application through the DfE Data Sharing Service. Approved data is made available via the ONS Secure Research Service (SRS), so researchers must hold ONS Accredited Researcher status to access it.</t>
-  </si>
-  <si>
-    <t>EYFSP, KS1 and KS2 attainment data are missing for pupils who attended independent or non-state schools, as these schools do not submit statutory assessment returns.
-The NPD school census includes only state-funded pupils. Independent schools do not provide pupil-level characteristics, even though they complete an annual census.</t>
-  </si>
-  <si>
     <t>Higher Education Statistics Agency (HESA)</t>
   </si>
   <si>
@@ -82,72 +52,54 @@
     <t>Subject studied, mode of study, award and degree classification, postcode, employment status, and occupation.</t>
   </si>
   <si>
-    <t>Student Record (1994/1995 to 2023/24).
-Graduate Outcomes Survey from 2017/2018 to 2023/24 (replaced the Destinations of Leavers from Higher Education survey, which ran from 2002/03 to 2016/17).
-Aggregate Offshore record (2007/08 to 2023/24)</t>
-  </si>
-  <si>
-    <t>Individual level and Provider level (for aggregate offshore record)</t>
-  </si>
-  <si>
-    <t>Managed by Jisc. Access requires organisational approval, a data-sharing agreement and a clear public-benefit rationale. HESA data can be accessed through HEAT (for member institutions), via LEO linkages (for specific variables), via institutional data-sharing agreements, or by submitting a direct data request to Jisc.</t>
-  </si>
-  <si>
-    <t>HESA primarily covers recognised HE courses at publicly funded HE providers. It does not comprehensively capture learners in sub-degree higher-level courses (e.g., HNCs/HNDs) that are often delivered in FE colleges. This can bias analyses toward traditional university pathways and underrepresent vocational/technical learners, staged FE-to-HE progression routes, mature learners, and other disadvantaged groups more likely to follow Level 4/5 routes.</t>
-  </si>
-  <si>
     <t>Longitudinal Education Outcomes (LEO)</t>
   </si>
   <si>
-    <t>Individuals who have enrolled in the English education system</t>
-  </si>
-  <si>
     <t>Employment status, earnings, benefit claims, sector of employment, type and size of organisation.</t>
   </si>
   <si>
-    <t>Employment (HMRC PAYE) available (1997/199 to 2020/21)
-Benefits (1999/00 to 2020/21)
-HESA (2004/05 to 2019/20)
-NPD (2001/02 to 2020/21, with earlier collections subject to the dataset) 
-IDBR Enterprise (2004/05 to 2020/21)
-UCAS (2007/08 to 2020/21)
-Furlough data (CJRS and SEISS available for 2020/21.
-Individual Learner records (2002/03 to 2020/21)</t>
-  </si>
-  <si>
     <t>Individual-level</t>
   </si>
   <si>
-    <t>Managed by the ONS. Access is highly restricted and requires submitting an the Project Accreditation Service (PASS). Access requires ONS Accredited Researcher status. Data linking is performed by data owners, not researchers. Only pseudonymised, pre-linked extracts are accessible, under SRS conditions.</t>
-  </si>
-  <si>
-    <t>All datasets included in the LEO can be linked at the individual level to each other, but no other individual-level data can be linked to LEO.
-LEO cannot track earnings for graduates who work or live outside the UK, because HMRC tax records only cover UK-based taxable income. As a result, individuals emigrating or working abroad are excluded from earnings data, which can bias results for highly mobile groups.</t>
-  </si>
-  <si>
     <t>Universities and Colleges Admissions Service (UCAS</t>
   </si>
   <si>
     <t>Applicants to higher education in the UK.</t>
   </si>
   <si>
-    <t>Applicant domicile, provider tariff band, achieved or predicted qualification points/grades, acceptance route, number of offers or choices, and year of entry</t>
-  </si>
-  <si>
-    <t>Available from 2007 to 2024/25.</t>
-  </si>
-  <si>
-    <t>Individual level, by stage of the application cycle</t>
-  </si>
-  <si>
-    <t>Managed by UCAS. Access is available through publicly released aggregated datasets, the UCAS EXACT Service for individual-level data, the UCAS Outreach Evaluator for aggregated-level data, and, for specific variables, via the LEO dataset for 18-year-old English applicants from 2007/08 onwards.</t>
+    <t>Children who attended school in England.</t>
+  </si>
+  <si>
+    <t>Individuals who have enrolled in the English education system.</t>
+  </si>
+  <si>
+    <t>Applicant domicile, provider tariff band, achieved or predicted qualification points/grades, acceptance route, number of offers or choices, and year of entry.</t>
+  </si>
+  <si>
+    <t>Individual level and provider level (for aggregate offshore record).</t>
+  </si>
+  <si>
+    <t>Individual level, by stage of the application cycle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1997/98 to present (varies by component) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1994/95 to present (varies by component) </t>
+  </si>
+  <si>
+    <t>2007 to present.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Years available 
+</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -158,12 +110,6 @@
       <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Barlow"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -186,19 +132,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -418,127 +358,96 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultColWidth="23.81640625" defaultRowHeight="13" x14ac:dyDescent="0.6"/>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultColWidth="23.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="16384" width="23.81640625" style="3"/>
+    <col min="1" max="16384" width="23.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="14" x14ac:dyDescent="0.8">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" ht="27" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="54" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="81" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="40.5" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="40.5" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="224" x14ac:dyDescent="0.8">
-      <c r="A2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="C5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="238" x14ac:dyDescent="0.8">
-      <c r="A3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="1" t="s">
+      <c r="E5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="224" x14ac:dyDescent="0.8">
-      <c r="A4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="154" x14ac:dyDescent="0.8">
-      <c r="A5" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" s="2"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A6" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>